<commit_message>
genetics: pin wild stock as pure lines; F1 uniform, F2 segregates
Design decision: wild plants are homozygous pure lines, so a first
wild-x-wild cross is a uniform F1 and heritable variation emerges in the
F2 (hybrid x hybrid). Records the decision, notes it in the genetics part
and the Phase 0 plan, and cleans the sandbox spreadsheet's wild genotypes
to be fully homozygous (only the intended discrete recessives now carry).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NMcQZ57ME9A8pCjNremANB
</commit_message>
<xml_diff>
--- a/docs/poc/phase-0-genetics-sandbox.xlsx
+++ b/docs/poc/phase-0-genetics-sandbox.xlsx
@@ -1067,7 +1067,7 @@
         </is>
       </c>
       <c r="C5" s="6">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D5" s="6">
         <v>38</v>
@@ -1079,10 +1079,10 @@
         <v>38</v>
       </c>
       <c r="G5" s="6">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H5" s="6">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I5" s="6">
         <v>24</v>
@@ -1183,7 +1183,7 @@
         <v>48</v>
       </c>
       <c r="E6" s="6">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F6" s="6">
         <v>47</v>
@@ -1418,10 +1418,10 @@
         <v>13</v>
       </c>
       <c r="J8" s="6">
+        <v>13</v>
+      </c>
+      <c r="K8" s="6">
         <v>12</v>
-      </c>
-      <c r="K8" s="6">
-        <v>13</v>
       </c>
       <c r="L8" s="6">
         <v>12</v>
@@ -1650,10 +1650,10 @@
         <v>8</v>
       </c>
       <c r="N10" s="6">
+        <v>8</v>
+      </c>
+      <c r="O10" s="6">
         <v>7</v>
-      </c>
-      <c r="O10" s="6">
-        <v>8</v>
       </c>
       <c r="P10" s="6">
         <v>7</v>

</xml_diff>